<commit_message>
chore(mappa): aggiornamento manuale 2026-05-19-1346
</commit_message>
<xml_diff>
--- a/Roma_2027.xlsx
+++ b/Roma_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41075A34-69E0-474C-82BE-27188CE94C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D60E0CC-A2DC-4F18-8DC9-4B67EDE49B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{370BB6BA-2F30-4775-942F-04016D8D18C4}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4420" uniqueCount="1922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4422" uniqueCount="1924">
   <si>
     <t>Recensore</t>
   </si>
@@ -5805,6 +5805,12 @@
   </si>
   <si>
     <t>41.51116783711071, 12.741851017737611</t>
+  </si>
+  <si>
+    <t>41.8944379009184, 12.493778041993513</t>
+  </si>
+  <si>
+    <t>41.94435489991688, 12.469034833268445</t>
   </si>
 </sst>
 </file>
@@ -6083,7 +6089,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6288,9 +6294,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="9" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6768,7 +6771,7 @@
         <f>+H3+H4</f>
         <v>257</v>
       </c>
-      <c r="I5" s="69"/>
+      <c r="I5" s="9"/>
       <c r="J5" s="9"/>
       <c r="K5" s="9"/>
       <c r="L5" s="9"/>
@@ -11149,7 +11152,9 @@
       <c r="H45" s="48" t="s">
         <v>357</v>
       </c>
-      <c r="I45" s="48"/>
+      <c r="I45" s="68" t="s">
+        <v>1922</v>
+      </c>
       <c r="J45" s="47" t="s">
         <v>491</v>
       </c>
@@ -28485,7 +28490,9 @@
       <c r="H201" s="35" t="s">
         <v>357</v>
       </c>
-      <c r="I201" s="35"/>
+      <c r="I201" s="39" t="s">
+        <v>1923</v>
+      </c>
       <c r="J201" s="34" t="s">
         <v>1202</v>
       </c>
@@ -46872,7 +46879,7 @@
       <c r="H366" s="61" t="s">
         <v>357</v>
       </c>
-      <c r="I366" s="70" t="s">
+      <c r="I366" s="69" t="s">
         <v>1915</v>
       </c>
       <c r="J366" s="60" t="s">

</xml_diff>

<commit_message>
chore(mappa): aggiornamento manuale 2026-05-19-1406
</commit_message>
<xml_diff>
--- a/Roma_2027.xlsx
+++ b/Roma_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27AED4A-AF6C-4BDF-9A7F-F84F14C78373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05D5EC9-2EEC-441D-AFD6-5FF561E5AF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{370BB6BA-2F30-4775-942F-04016D8D18C4}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4426" uniqueCount="1928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4432" uniqueCount="1934">
   <si>
     <t>Recensore</t>
   </si>
@@ -5823,6 +5823,24 @@
   </si>
   <si>
     <t>41.89776107504589, 12.468759116941461</t>
+  </si>
+  <si>
+    <t>41.37728946359321, 13.737764537660487</t>
+  </si>
+  <si>
+    <t>41.82955701496672, 13.166111144621077</t>
+  </si>
+  <si>
+    <t>41.82857927673047, 13.143353525815082</t>
+  </si>
+  <si>
+    <t>41.80976549234967, 13.122920514770096</t>
+  </si>
+  <si>
+    <t>41.89472309055656, 12.474234812461015</t>
+  </si>
+  <si>
+    <t>41.89456883018618, 12.474274381610769</t>
   </si>
 </sst>
 </file>
@@ -15509,7 +15527,9 @@
         <v>698</v>
       </c>
       <c r="N84" s="17"/>
-      <c r="Q84" s="16"/>
+      <c r="Q84" s="20" t="s">
+        <v>1929</v>
+      </c>
       <c r="S84" s="1">
         <f t="shared" si="35"/>
         <v>0</v>
@@ -16508,7 +16528,9 @@
         <v>39</v>
       </c>
       <c r="N93" s="17"/>
-      <c r="Q93" s="16"/>
+      <c r="Q93" s="20" t="s">
+        <v>1931</v>
+      </c>
       <c r="S93" s="1">
         <f t="shared" si="47"/>
         <v>0</v>
@@ -22298,7 +22320,9 @@
       <c r="P145" s="38">
         <v>1</v>
       </c>
-      <c r="Q145" s="35"/>
+      <c r="Q145" s="35" t="s">
+        <v>1928</v>
+      </c>
       <c r="S145" s="1">
         <f t="shared" si="63"/>
         <v>0</v>
@@ -27299,7 +27323,9 @@
         <v>698</v>
       </c>
       <c r="N190" s="17"/>
-      <c r="Q190" s="16"/>
+      <c r="Q190" s="20" t="s">
+        <v>1930</v>
+      </c>
       <c r="S190" s="1">
         <f t="shared" si="63"/>
         <v>0</v>
@@ -48249,7 +48275,9 @@
       </c>
       <c r="O378" s="51"/>
       <c r="P378" s="51"/>
-      <c r="Q378" s="48"/>
+      <c r="Q378" s="48" t="s">
+        <v>1933</v>
+      </c>
       <c r="S378" s="1">
         <f t="shared" si="111"/>
         <v>1</v>
@@ -50582,7 +50610,9 @@
       </c>
       <c r="O399" s="51"/>
       <c r="P399" s="51"/>
-      <c r="Q399" s="48"/>
+      <c r="Q399" s="48" t="s">
+        <v>1932</v>
+      </c>
       <c r="S399" s="1">
         <f t="shared" si="139"/>
         <v>1</v>

</xml_diff>